<commit_message>
a fix hotter than a nuclear explosion
</commit_message>
<xml_diff>
--- a/02.04.2026.xlsx
+++ b/02.04.2026.xlsx
@@ -10,45 +10,57 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName localSheetId="0" name="_xlnm.Print_Area">Sheet1!$A$1:$B$16</definedName>
+    <definedName localSheetId="0" name="_xlnm.Print_Area">Sheet1!$A$1:$B$136</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+  <si>
+    <t>312580</t>
+  </si>
+  <si>
+    <t>Среднетемпературный режим (+2+6)</t>
+  </si>
+  <si>
+    <t>Наименование:</t>
+  </si>
+  <si>
+    <t>Охлаждённая продукция</t>
+  </si>
+  <si>
+    <t>Заказчик:</t>
+  </si>
+  <si>
+    <t>STEAK HOME</t>
+  </si>
+  <si>
+    <t>Получатель:</t>
+  </si>
+  <si>
+    <t>Аксарин Павел</t>
+  </si>
+  <si>
+    <t>Вх. накладная:</t>
+  </si>
+  <si>
+    <t>Адрес доставки:</t>
+  </si>
+  <si>
+    <t>Россия, Московская область, муниципальный округ Истра, КП Гринфилд, д. 22</t>
+  </si>
+  <si>
+    <t>(1 из 1)</t>
+  </si>
   <si>
     <t>312581</t>
   </si>
   <si>
-    <t>Среднетемпературный режим (+2+6)</t>
-  </si>
-  <si>
-    <t>Наименование:</t>
-  </si>
-  <si>
-    <t>Охлаждённая продукция</t>
-  </si>
-  <si>
-    <t>Заказчик:</t>
-  </si>
-  <si>
-    <t>STEAK HOME</t>
-  </si>
-  <si>
-    <t>Получатель:</t>
-  </si>
-  <si>
     <t>Доманов Максим</t>
   </si>
   <si>
-    <t>Вх. накладная:</t>
-  </si>
-  <si>
-    <t>Адрес доставки:</t>
-  </si>
-  <si>
     <t>Россия, Москва, проспект Мира, д. 188Бк1</t>
   </si>
   <si>
@@ -62,6 +74,108 @@
   </si>
   <si>
     <t>(2 из 2)</t>
+  </si>
+  <si>
+    <t>312582</t>
+  </si>
+  <si>
+    <t>Ивашкина Елена</t>
+  </si>
+  <si>
+    <t>Москва, улица Академика Виноградова, д. 5</t>
+  </si>
+  <si>
+    <t>312583</t>
+  </si>
+  <si>
+    <t>Иванов Михаил</t>
+  </si>
+  <si>
+    <t>Москва, Профсоюзная улица, д. 125к1</t>
+  </si>
+  <si>
+    <t>312584</t>
+  </si>
+  <si>
+    <t>Константин</t>
+  </si>
+  <si>
+    <t>Московская область, городской округ Красногорск, посёлок дачного хозяйства Архангельское, 7-я линия</t>
+  </si>
+  <si>
+    <t>(1 из 3)</t>
+  </si>
+  <si>
+    <t>(2 из 3)</t>
+  </si>
+  <si>
+    <t>(3 из 3)</t>
+  </si>
+  <si>
+    <t>312585</t>
+  </si>
+  <si>
+    <t>Александр</t>
+  </si>
+  <si>
+    <t>Москва, Балаклавский проспект, д. 15</t>
+  </si>
+  <si>
+    <t>312586</t>
+  </si>
+  <si>
+    <t>312587</t>
+  </si>
+  <si>
+    <t>Иванов Александр</t>
+  </si>
+  <si>
+    <t>Москва, Славянская площадь, д. 4с3</t>
+  </si>
+  <si>
+    <t>312588</t>
+  </si>
+  <si>
+    <t>Гайнар Ирина</t>
+  </si>
+  <si>
+    <t>Москва, улица Маршала Тухачевского, д. 32к2</t>
+  </si>
+  <si>
+    <t>312589</t>
+  </si>
+  <si>
+    <t>Жаглин Антон</t>
+  </si>
+  <si>
+    <t>Московская область, Химки, микрорайон Сходня, Овражная улица, д. 24к2</t>
+  </si>
+  <si>
+    <t>312590</t>
+  </si>
+  <si>
+    <t>Варвара</t>
+  </si>
+  <si>
+    <t>Москва, улица Гризодубовой, д. 4к2</t>
+  </si>
+  <si>
+    <t>312591</t>
+  </si>
+  <si>
+    <t>Крылов Николай</t>
+  </si>
+  <si>
+    <t>Московская область, Ленинский городской округ, деревня Суханово, жилой комплекс Суханово Парк, д. 92</t>
+  </si>
+  <si>
+    <t>312592</t>
+  </si>
+  <si>
+    <t>Богатырев Вадим</t>
+  </si>
+  <si>
+    <t>Москва, улица Маршала Соколовского, д. 5</t>
   </si>
 </sst>
 </file>
@@ -180,7 +294,487 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 4" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 7" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 8" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 9" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 10" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 11" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 12" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 13" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 14" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>104</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 15" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>112</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 16" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>120</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 17" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1333500" cy="523875"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>128</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1333500" cy="523875"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 18" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -523,13 +1117,13 @@
     </row>
     <row r="9" ht="62" customHeight="true">
       <c r="A9" s="3" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B9" s="3"/>
     </row>
     <row r="10" ht="20" customHeight="true">
       <c r="A10" s="3" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B10" s="3"/>
     </row>
@@ -538,7 +1132,7 @@
         <v>2</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" ht="12" customHeight="true">
@@ -554,7 +1148,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="true">
@@ -562,7 +1156,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -570,24 +1164,924 @@
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" ht="12" customHeight="true">
       <c r="B16" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" ht="62" customHeight="true">
+      <c r="A17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="3"/>
+    </row>
+    <row r="18" ht="20" customHeight="true">
+      <c r="A18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3"/>
+    </row>
+    <row r="19" ht="12" customHeight="true">
+      <c r="A19" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" ht="12" customHeight="true">
+      <c r="A20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" ht="12" customHeight="true">
+      <c r="A21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" ht="12" customHeight="true">
+      <c r="A22" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>14</v>
       </c>
     </row>
+    <row r="24" ht="12" customHeight="true">
+      <c r="B24" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" ht="62" customHeight="true">
+      <c r="A25" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="3"/>
+    </row>
+    <row r="26" ht="20" customHeight="true">
+      <c r="A26" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="3"/>
+    </row>
+    <row r="27" ht="12" customHeight="true">
+      <c r="A27" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" ht="12" customHeight="true">
+      <c r="A28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" ht="12" customHeight="true">
+      <c r="A29" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" ht="12" customHeight="true">
+      <c r="A30" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" ht="12" customHeight="true">
+      <c r="B32" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" ht="62" customHeight="true">
+      <c r="A33" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B33" s="3"/>
+    </row>
+    <row r="34" ht="20" customHeight="true">
+      <c r="A34" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34" s="3"/>
+    </row>
+    <row r="35" ht="12" customHeight="true">
+      <c r="A35" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" ht="12" customHeight="true">
+      <c r="A36" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" ht="12" customHeight="true">
+      <c r="A37" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="38" ht="12" customHeight="true">
+      <c r="A38" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" ht="12" customHeight="true">
+      <c r="B40" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" ht="62" customHeight="true">
+      <c r="A41" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B41" s="3"/>
+    </row>
+    <row r="42" ht="20" customHeight="true">
+      <c r="A42" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B42" s="3"/>
+    </row>
+    <row r="43" ht="12" customHeight="true">
+      <c r="A43" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" ht="12" customHeight="true">
+      <c r="A44" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" ht="12" customHeight="true">
+      <c r="A45" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" ht="12" customHeight="true">
+      <c r="A46" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="48" ht="12" customHeight="true">
+      <c r="B48" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="49" ht="62" customHeight="true">
+      <c r="A49" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B49" s="3"/>
+    </row>
+    <row r="50" ht="20" customHeight="true">
+      <c r="A50" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50" s="3"/>
+    </row>
+    <row r="51" ht="12" customHeight="true">
+      <c r="A51" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" ht="12" customHeight="true">
+      <c r="A52" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" ht="12" customHeight="true">
+      <c r="A53" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="54" ht="12" customHeight="true">
+      <c r="A54" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="56" ht="12" customHeight="true">
+      <c r="B56" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="57" ht="62" customHeight="true">
+      <c r="A57" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B57" s="3"/>
+    </row>
+    <row r="58" ht="20" customHeight="true">
+      <c r="A58" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B58" s="3"/>
+    </row>
+    <row r="59" ht="12" customHeight="true">
+      <c r="A59" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60" ht="12" customHeight="true">
+      <c r="A60" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="61" ht="12" customHeight="true">
+      <c r="A61" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="62" ht="12" customHeight="true">
+      <c r="A62" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="64" ht="12" customHeight="true">
+      <c r="B64" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="65" ht="62" customHeight="true">
+      <c r="A65" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B65" s="3"/>
+    </row>
+    <row r="66" ht="20" customHeight="true">
+      <c r="A66" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B66" s="3"/>
+    </row>
+    <row r="67" ht="12" customHeight="true">
+      <c r="A67" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="68" ht="12" customHeight="true">
+      <c r="A68" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="69" ht="12" customHeight="true">
+      <c r="A69" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="70" ht="12" customHeight="true">
+      <c r="A70" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="72" ht="12" customHeight="true">
+      <c r="B72" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="73" ht="62" customHeight="true">
+      <c r="A73" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B73" s="3"/>
+    </row>
+    <row r="74" ht="20" customHeight="true">
+      <c r="A74" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B74" s="3"/>
+    </row>
+    <row r="75" ht="12" customHeight="true">
+      <c r="A75" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" ht="12" customHeight="true">
+      <c r="A76" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77" ht="12" customHeight="true">
+      <c r="A77" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="78" ht="12" customHeight="true">
+      <c r="A78" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80" ht="12" customHeight="true">
+      <c r="B80" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="81" ht="62" customHeight="true">
+      <c r="A81" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B81" s="3"/>
+    </row>
+    <row r="82" ht="20" customHeight="true">
+      <c r="A82" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B82" s="3"/>
+    </row>
+    <row r="83" ht="12" customHeight="true">
+      <c r="A83" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="84" ht="12" customHeight="true">
+      <c r="A84" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="85" ht="12" customHeight="true">
+      <c r="A85" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="86" ht="12" customHeight="true">
+      <c r="A86" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="88" ht="12" customHeight="true">
+      <c r="B88" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="89" ht="62" customHeight="true">
+      <c r="A89" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B89" s="3"/>
+    </row>
+    <row r="90" ht="20" customHeight="true">
+      <c r="A90" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B90" s="3"/>
+    </row>
+    <row r="91" ht="12" customHeight="true">
+      <c r="A91" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="92" ht="12" customHeight="true">
+      <c r="A92" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="93" ht="12" customHeight="true">
+      <c r="A93" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="94" ht="12" customHeight="true">
+      <c r="A94" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="96" ht="12" customHeight="true">
+      <c r="B96" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="97" ht="62" customHeight="true">
+      <c r="A97" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B97" s="3"/>
+    </row>
+    <row r="98" ht="20" customHeight="true">
+      <c r="A98" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B98" s="3"/>
+    </row>
+    <row r="99" ht="12" customHeight="true">
+      <c r="A99" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="100" ht="12" customHeight="true">
+      <c r="A100" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101" ht="12" customHeight="true">
+      <c r="A101" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="102" ht="12" customHeight="true">
+      <c r="A102" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="104" ht="12" customHeight="true">
+      <c r="B104" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="105" ht="62" customHeight="true">
+      <c r="A105" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B105" s="3"/>
+    </row>
+    <row r="106" ht="20" customHeight="true">
+      <c r="A106" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B106" s="3"/>
+    </row>
+    <row r="107" ht="12" customHeight="true">
+      <c r="A107" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="108" ht="12" customHeight="true">
+      <c r="A108" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="109" ht="12" customHeight="true">
+      <c r="A109" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="110" ht="12" customHeight="true">
+      <c r="A110" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="112" ht="12" customHeight="true">
+      <c r="B112" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="113" ht="62" customHeight="true">
+      <c r="A113" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B113" s="3"/>
+    </row>
+    <row r="114" ht="20" customHeight="true">
+      <c r="A114" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B114" s="3"/>
+    </row>
+    <row r="115" ht="12" customHeight="true">
+      <c r="A115" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="116" ht="12" customHeight="true">
+      <c r="A116" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="117" ht="12" customHeight="true">
+      <c r="A117" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="118" ht="12" customHeight="true">
+      <c r="A118" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="120" ht="12" customHeight="true">
+      <c r="B120" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="121" ht="62" customHeight="true">
+      <c r="A121" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B121" s="3"/>
+    </row>
+    <row r="122" ht="20" customHeight="true">
+      <c r="A122" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B122" s="3"/>
+    </row>
+    <row r="123" ht="12" customHeight="true">
+      <c r="A123" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="124" ht="12" customHeight="true">
+      <c r="A124" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="125" ht="12" customHeight="true">
+      <c r="A125" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="126" ht="12" customHeight="true">
+      <c r="A126" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="128" ht="12" customHeight="true">
+      <c r="B128" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="129" ht="62" customHeight="true">
+      <c r="A129" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B129" s="3"/>
+    </row>
+    <row r="130" ht="20" customHeight="true">
+      <c r="A130" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B130" s="3"/>
+    </row>
+    <row r="131" ht="12" customHeight="true">
+      <c r="A131" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="132" ht="12" customHeight="true">
+      <c r="A132" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="133" ht="12" customHeight="true">
+      <c r="A133" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="134" ht="12" customHeight="true">
+      <c r="A134" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="136" ht="12" customHeight="true">
+      <c r="B136" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="34">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="A82:B82"/>
+    <mergeCell ref="A89:B89"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="A97:B97"/>
+    <mergeCell ref="A98:B98"/>
+    <mergeCell ref="A105:B105"/>
+    <mergeCell ref="A106:B106"/>
+    <mergeCell ref="A113:B113"/>
+    <mergeCell ref="A114:B114"/>
+    <mergeCell ref="A121:B121"/>
+    <mergeCell ref="A122:B122"/>
+    <mergeCell ref="A129:B129"/>
+    <mergeCell ref="A130:B130"/>
   </mergeCells>
-  <rowBreaks count="2" manualBreakCount="2">
+  <rowBreaks count="17" manualBreakCount="17">
     <brk id="8" max="16383" man="true"/>
     <brk id="16" max="16383" man="true"/>
+    <brk id="24" max="16383" man="true"/>
+    <brk id="32" max="16383" man="true"/>
+    <brk id="40" max="16383" man="true"/>
+    <brk id="48" max="16383" man="true"/>
+    <brk id="56" max="16383" man="true"/>
+    <brk id="64" max="16383" man="true"/>
+    <brk id="72" max="16383" man="true"/>
+    <brk id="80" max="16383" man="true"/>
+    <brk id="88" max="16383" man="true"/>
+    <brk id="96" max="16383" man="true"/>
+    <brk id="104" max="16383" man="true"/>
+    <brk id="112" max="16383" man="true"/>
+    <brk id="120" max="16383" man="true"/>
+    <brk id="128" max="16383" man="true"/>
+    <brk id="136" max="16383" man="true"/>
   </rowBreaks>
   <colBreaks/>
   <drawing r:id="rId1"/>

</xml_diff>